<commit_message>
Made mobile friendly. Add eye growth. Multipliers now stack
</commit_message>
<xml_diff>
--- a/public/monster_rewards.xlsx
+++ b/public/monster_rewards.xlsx
@@ -412,7 +412,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -420,7 +420,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -428,7 +428,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>50</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5">
@@ -436,7 +436,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>75</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6">
@@ -444,7 +444,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>100</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7">
@@ -452,7 +452,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>125</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8">
@@ -460,7 +460,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>150</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9">
@@ -468,7 +468,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>175</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10">
@@ -476,7 +476,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>200</v>
+        <v>175</v>
       </c>
     </row>
     <row r="11">
@@ -484,7 +484,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>250</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>